<commit_message>
add fields penalty_fee for equipment
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_matrix_dot2.xlsx
+++ b/docs/SLMS2026_import_matrix_dot2.xlsx
@@ -404,9 +404,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
-  <cols>
-    <col min="1" max="1" width="41.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -443,17 +440,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I15"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -804,11 +790,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C22"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1014,11 +995,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C9"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="23.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1129,15 +1105,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G13"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1448,13 +1415,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E11"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="23.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1652,20 +1612,21 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="17.83203125" customWidth="1"/>
-    <col min="9" max="9" width="21.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
-    <col min="11" max="11" width="21.83203125" customWidth="1"/>
-    <col min="12" max="12" width="19.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="21.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" customWidth="1"/>
+    <col min="10" max="10" width="23.83203125" customWidth="1"/>
+    <col min="11" max="11" width="19.83203125" customWidth="1"/>
+    <col min="12" max="12" width="29.83203125" customWidth="1"/>
+    <col min="13" max="13" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1703,6 +1664,9 @@
         <v>Ngày hết bảo hành</v>
       </c>
       <c r="L1" t="str">
+        <v>Giá phạt hết bảo hành (VNĐ)</v>
+      </c>
+      <c r="M1" t="str">
         <v>Ghi chú lắp đặt</v>
       </c>
     </row>
@@ -1740,7 +1704,10 @@
       <c r="K2" t="str">
         <v>2028-04-30</v>
       </c>
-      <c r="L2" t="str">
+      <c r="L2">
+        <v>3000000</v>
+      </c>
+      <c r="M2" t="str">
         <v/>
       </c>
     </row>
@@ -1778,7 +1745,10 @@
       <c r="K3" t="str">
         <v>2028-04-30</v>
       </c>
-      <c r="L3" t="str">
+      <c r="L3">
+        <v>2000000</v>
+      </c>
+      <c r="M3" t="str">
         <v/>
       </c>
     </row>
@@ -1816,7 +1786,10 @@
       <c r="K4" t="str">
         <v>2029-05-31</v>
       </c>
-      <c r="L4" t="str">
+      <c r="L4">
+        <v>3500000</v>
+      </c>
+      <c r="M4" t="str">
         <v/>
       </c>
     </row>
@@ -1854,7 +1827,10 @@
       <c r="K5" t="str">
         <v>2027-05-31</v>
       </c>
-      <c r="L5" t="str">
+      <c r="L5">
+        <v>800000</v>
+      </c>
+      <c r="M5" t="str">
         <v/>
       </c>
     </row>
@@ -1892,7 +1868,10 @@
       <c r="K6" t="str">
         <v>2027-06-28</v>
       </c>
-      <c r="L6" t="str">
+      <c r="L6">
+        <v>1500000</v>
+      </c>
+      <c r="M6" t="str">
         <v>TB mới phòng 101</v>
       </c>
     </row>
@@ -1930,7 +1909,10 @@
       <c r="K7" t="str">
         <v>2028-06-28</v>
       </c>
-      <c r="L7" t="str">
+      <c r="L7">
+        <v>2500000</v>
+      </c>
+      <c r="M7" t="str">
         <v>TB mới phòng 102</v>
       </c>
     </row>
@@ -1968,7 +1950,10 @@
       <c r="K8" t="str">
         <v>2027-06-28</v>
       </c>
-      <c r="L8" t="str">
+      <c r="L8">
+        <v>700000</v>
+      </c>
+      <c r="M8" t="str">
         <v>TB mới phòng 103</v>
       </c>
     </row>
@@ -2006,7 +1991,10 @@
       <c r="K9" t="str">
         <v>2027-07-28</v>
       </c>
-      <c r="L9" t="str">
+      <c r="L9">
+        <v>1500000</v>
+      </c>
+      <c r="M9" t="str">
         <v>TB mới phòng 101</v>
       </c>
     </row>
@@ -2044,7 +2032,10 @@
       <c r="K10" t="str">
         <v>2028-07-28</v>
       </c>
-      <c r="L10" t="str">
+      <c r="L10">
+        <v>2500000</v>
+      </c>
+      <c r="M10" t="str">
         <v>TB mới phòng 102</v>
       </c>
     </row>
@@ -2082,13 +2073,16 @@
       <c r="K11" t="str">
         <v>2027-07-28</v>
       </c>
-      <c r="L11" t="str">
+      <c r="L11">
+        <v>700000</v>
+      </c>
+      <c r="M11" t="str">
         <v>TB mới phòng 103</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>